<commit_message>
Lab 4: Add TaskDetailPage with status update and delete
</commit_message>
<xml_diff>
--- a/Робота/ЄДБО_Збір.xlsx
+++ b/Робота/ЄДБО_Збір.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Всякие документы\Sem_2\Робота\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FED4A235-E39C-4D81-97F2-E980C8A62379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D884F05-A56A-4237-AC41-EFC490E5096B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30450" yWindow="3360" windowWidth="21600" windowHeight="11385" xr2:uid="{961233AC-788E-4C66-80C9-0CCA6031536C}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{961233AC-788E-4C66-80C9-0CCA6031536C}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="32">
   <si>
     <t>№</t>
   </si>
@@ -127,6 +127,9 @@
   </si>
   <si>
     <t>+</t>
+  </si>
+  <si>
+    <t>Бічевий Матівй</t>
   </si>
 </sst>
 </file>
@@ -522,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59A5E092-B5E4-4073-8AD7-1A49634A03DA}">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" customWidth="1"/>
@@ -546,7 +549,9 @@
       <c r="B2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="5"/>
+      <c r="C2" s="5" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="3" spans="1:3" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
@@ -555,7 +560,9 @@
       <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="5"/>
+      <c r="C3" s="5" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="4" spans="1:3" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
@@ -564,7 +571,9 @@
       <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="5"/>
+      <c r="C4" s="5" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="5" spans="1:3" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
@@ -584,7 +593,9 @@
       <c r="B6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="5"/>
+      <c r="C6" s="5" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="7" spans="1:3" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
@@ -626,7 +637,9 @@
       <c r="B10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="5"/>
+      <c r="C10" s="5" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="11" spans="1:3" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
@@ -646,7 +659,9 @@
       <c r="B12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="5"/>
+      <c r="C12" s="5" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="13" spans="1:3" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
@@ -726,7 +741,9 @@
       <c r="B20" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="5"/>
+      <c r="C20" s="5" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="21" spans="1:3" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
@@ -762,7 +779,9 @@
       <c r="B24" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C24" s="5"/>
+      <c r="C24" s="5" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="25" spans="1:3" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
@@ -771,7 +790,9 @@
       <c r="B25" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C25" s="5"/>
+      <c r="C25" s="5" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="26" spans="1:3" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
@@ -800,7 +821,9 @@
       <c r="B28" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C28" s="5"/>
+      <c r="C28" s="5" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="29" spans="1:3" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
@@ -818,7 +841,9 @@
       <c r="B30" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C30" s="5"/>
+      <c r="C30" s="5" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="31" spans="1:3" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
@@ -827,7 +852,20 @@
       <c r="B31" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C31" s="5"/>
+      <c r="C31" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="3">
+        <v>31</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>